<commit_message>
feeding cash data till june
</commit_message>
<xml_diff>
--- a/src/app/api/dashboard/data_entry/Cash_Till_June.xlsx
+++ b/src/app/api/dashboard/data_entry/Cash_Till_June.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/9f13febc4eefe037/Documents/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="8" documentId="8_{5E607731-EE77-444E-B1DE-FC58CE38B93F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{7F2F9593-5F72-43AE-AE65-0C39D357F4CA}"/>
+  <xr:revisionPtr revIDLastSave="9" documentId="8_{5E607731-EE77-444E-B1DE-FC58CE38B93F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{9DD1B445-2D7C-4D2B-AC7B-C19C9E84F445}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{8B043C64-D4CE-4BC2-B3E8-A1907E08430C}"/>
   </bookViews>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="422" uniqueCount="188">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="344" uniqueCount="157">
   <si>
     <t>phone</t>
   </si>
@@ -103,99 +103,6 @@
   </si>
   <si>
     <t>H.NO. 2-4-1247/4/3, T V TOWER</t>
-  </si>
-  <si>
-    <t>N HARINI</t>
-  </si>
-  <si>
-    <t>BANGALORE</t>
-  </si>
-  <si>
-    <t>KARNATAKA</t>
-  </si>
-  <si>
-    <t>DIVYA SURYA MAHENDER</t>
-  </si>
-  <si>
-    <t>H.NO. GOPALPURAM, USHODAYA COLONY,</t>
-  </si>
-  <si>
-    <t>V RAJARAM</t>
-  </si>
-  <si>
-    <t>GOLI DIWAKAR BHARATHI</t>
-  </si>
-  <si>
-    <t>FLAT NO 510, GOPALAN GRANDE APARTMENT, NAIMNAGAR</t>
-  </si>
-  <si>
-    <t>K RAVI KUMAR</t>
-  </si>
-  <si>
-    <t>H.NO. 19-42/1/A, NARSAMPET</t>
-  </si>
-  <si>
-    <t>S YADARARI</t>
-  </si>
-  <si>
-    <t>H.NO. 15-193/A/A, THORRUR</t>
-  </si>
-  <si>
-    <t>OM PRAKASH</t>
-  </si>
-  <si>
-    <t>H.NO. FLAT 510, GOPALAN GRANDE APARTMENT, NAIMNAGAR</t>
-  </si>
-  <si>
-    <t>P CHIRANJEEVI</t>
-  </si>
-  <si>
-    <t>DHARMASAGAR,</t>
-  </si>
-  <si>
-    <t>MUDDASANI VIJAYA</t>
-  </si>
-  <si>
-    <t>H.NO. 55-2-585, SATYA SAI COLONY,</t>
-  </si>
-  <si>
-    <t>NAGA PARAM KUMAR</t>
-  </si>
-  <si>
-    <t>H.NO. 101, VSR TOWERS, TEACHERS COLONY, PHASE II,</t>
-  </si>
-  <si>
-    <t>HARI</t>
-  </si>
-  <si>
-    <t>NAGENDER</t>
-  </si>
-  <si>
-    <t xml:space="preserve">WARANGAL </t>
-  </si>
-  <si>
-    <t>SOUJANYA</t>
-  </si>
-  <si>
-    <t>AKRUTHI, OPP TO PAIDPALLY X ROAD</t>
-  </si>
-  <si>
-    <t>SREE NITHITA</t>
-  </si>
-  <si>
-    <t>H.NO. 7-1-47/4/503, RATNDEEP RESIDENCY</t>
-  </si>
-  <si>
-    <t>B VARSHA</t>
-  </si>
-  <si>
-    <t xml:space="preserve">H.NO. 4-2-138, </t>
-  </si>
-  <si>
-    <t>SIDDHARTHA</t>
-  </si>
-  <si>
-    <t>URSUGUTTA, KARIMABAD,</t>
   </si>
   <si>
     <t>KRISHNA</t>
@@ -962,7 +869,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6179F6AC-DDA8-4254-81E8-FA076EAF5481}">
-  <dimension ref="A1:L84"/>
+  <dimension ref="A1:L68"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="11.88671875" bestFit="1" customWidth="1"/>
@@ -999,10 +906,10 @@
         <v>5</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>187</v>
+        <v>156</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>186</v>
+        <v>155</v>
       </c>
       <c r="I1" s="1" t="s">
         <v>6</v>
@@ -1019,100 +926,103 @@
     </row>
     <row r="2" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A2">
-        <v>9980056611</v>
+        <v>7997093302</v>
       </c>
       <c r="B2" t="s">
         <v>23</v>
       </c>
       <c r="C2">
-        <v>500</v>
+        <v>520</v>
       </c>
       <c r="D2" t="s">
         <v>10</v>
       </c>
       <c r="G2">
-        <v>2734</v>
+        <v>2783</v>
       </c>
       <c r="H2">
-        <v>46150</v>
+        <v>46158</v>
       </c>
       <c r="I2" t="s">
         <v>24</v>
       </c>
       <c r="J2" t="s">
-        <v>24</v>
+        <v>11</v>
       </c>
       <c r="K2" t="s">
-        <v>25</v>
+        <v>12</v>
+      </c>
+      <c r="L2">
+        <v>506142</v>
       </c>
     </row>
     <row r="3" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A3">
-        <v>9440086356</v>
+        <v>9704476844</v>
       </c>
       <c r="B3" t="s">
+        <v>25</v>
+      </c>
+      <c r="C3">
+        <v>520</v>
+      </c>
+      <c r="D3" t="s">
+        <v>10</v>
+      </c>
+      <c r="G3">
+        <v>2782</v>
+      </c>
+      <c r="H3">
+        <v>46158</v>
+      </c>
+      <c r="I3" t="s">
         <v>26</v>
       </c>
-      <c r="C3">
-        <v>210</v>
-      </c>
-      <c r="D3" t="s">
-        <v>10</v>
-      </c>
-      <c r="G3">
-        <v>2735</v>
-      </c>
-      <c r="H3">
-        <v>46150</v>
-      </c>
-      <c r="I3" t="s">
-        <v>27</v>
-      </c>
       <c r="J3" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="K3" t="s">
         <v>12</v>
       </c>
       <c r="L3">
-        <v>506001</v>
+        <v>506002</v>
       </c>
     </row>
     <row r="4" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A4">
-        <v>9849502796</v>
+        <v>9849502601</v>
       </c>
       <c r="B4" t="s">
+        <v>27</v>
+      </c>
+      <c r="C4">
+        <v>501</v>
+      </c>
+      <c r="D4" t="s">
+        <v>10</v>
+      </c>
+      <c r="G4">
+        <v>2789</v>
+      </c>
+      <c r="H4">
+        <v>46159</v>
+      </c>
+      <c r="I4" t="s">
         <v>28</v>
       </c>
-      <c r="C4">
-        <v>516</v>
-      </c>
-      <c r="D4" t="s">
-        <v>10</v>
-      </c>
-      <c r="G4">
-        <v>2741</v>
-      </c>
-      <c r="H4">
-        <v>46151</v>
-      </c>
-      <c r="I4" t="s">
-        <v>13</v>
-      </c>
       <c r="J4" t="s">
-        <v>13</v>
+        <v>18</v>
       </c>
       <c r="K4" t="s">
         <v>12</v>
       </c>
       <c r="L4">
-        <v>506001</v>
+        <v>506003</v>
       </c>
     </row>
     <row r="5" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A5">
-        <v>9290099905</v>
+        <v>9959715373</v>
       </c>
       <c r="B5" t="s">
         <v>29</v>
@@ -1124,27 +1034,27 @@
         <v>10</v>
       </c>
       <c r="G5">
-        <v>2750</v>
+        <v>2781</v>
       </c>
       <c r="H5">
-        <v>46152</v>
+        <v>46160</v>
       </c>
       <c r="I5" t="s">
         <v>30</v>
       </c>
       <c r="J5" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="K5" t="s">
         <v>12</v>
       </c>
       <c r="L5">
-        <v>506001</v>
+        <v>506002</v>
       </c>
     </row>
     <row r="6" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A6">
-        <v>8886888398</v>
+        <v>9492781734</v>
       </c>
       <c r="B6" t="s">
         <v>31</v>
@@ -1156,71 +1066,74 @@
         <v>10</v>
       </c>
       <c r="G6">
-        <v>2744</v>
+        <v>2790</v>
       </c>
       <c r="H6">
-        <v>46152</v>
+        <v>46160</v>
       </c>
       <c r="I6" t="s">
         <v>32</v>
       </c>
       <c r="J6" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="K6" t="s">
         <v>12</v>
       </c>
       <c r="L6">
-        <v>506330</v>
+        <v>506001</v>
       </c>
     </row>
     <row r="7" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A7">
-        <v>9182932142</v>
+        <v>9705036449</v>
       </c>
       <c r="B7" t="s">
         <v>33</v>
       </c>
       <c r="C7">
-        <v>511</v>
+        <v>500</v>
       </c>
       <c r="D7" t="s">
         <v>10</v>
       </c>
       <c r="G7">
-        <v>2743</v>
+        <v>2793</v>
       </c>
       <c r="H7">
-        <v>46152</v>
+        <v>46163</v>
       </c>
       <c r="I7" t="s">
         <v>34</v>
       </c>
+      <c r="J7" t="s">
+        <v>19</v>
+      </c>
       <c r="K7" t="s">
         <v>12</v>
       </c>
       <c r="L7">
-        <v>506213</v>
+        <v>506169</v>
       </c>
     </row>
     <row r="8" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A8">
-        <v>9959877803</v>
+        <v>9030936319</v>
       </c>
       <c r="B8" t="s">
         <v>35</v>
       </c>
       <c r="C8">
-        <v>520</v>
+        <v>516</v>
       </c>
       <c r="D8" t="s">
         <v>10</v>
       </c>
       <c r="G8">
-        <v>2757</v>
+        <v>2794</v>
       </c>
       <c r="H8">
-        <v>46152</v>
+        <v>46164</v>
       </c>
       <c r="I8" t="s">
         <v>36</v>
@@ -1237,307 +1150,313 @@
     </row>
     <row r="9" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A9">
-        <v>7981526312</v>
+        <v>8985635919</v>
       </c>
       <c r="B9" t="s">
         <v>37</v>
       </c>
       <c r="C9">
-        <v>500</v>
+        <v>520</v>
       </c>
       <c r="D9" t="s">
         <v>10</v>
       </c>
       <c r="G9">
-        <v>2760</v>
+        <v>2795</v>
       </c>
       <c r="H9">
-        <v>46152</v>
+        <v>46165</v>
       </c>
       <c r="I9" t="s">
         <v>38</v>
       </c>
       <c r="J9" t="s">
-        <v>13</v>
+        <v>20</v>
       </c>
       <c r="K9" t="s">
         <v>12</v>
       </c>
       <c r="L9">
-        <v>506143</v>
+        <v>506344</v>
       </c>
     </row>
     <row r="10" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A10">
-        <v>9849733381</v>
+        <v>8328376765</v>
       </c>
       <c r="B10" t="s">
         <v>39</v>
       </c>
       <c r="C10">
-        <v>3000</v>
+        <v>500</v>
       </c>
       <c r="D10" t="s">
         <v>10</v>
       </c>
       <c r="G10">
-        <v>2762</v>
+        <v>2803</v>
       </c>
       <c r="H10">
-        <v>46153</v>
+        <v>46166</v>
       </c>
       <c r="I10" t="s">
         <v>40</v>
       </c>
       <c r="J10" t="s">
-        <v>13</v>
+        <v>20</v>
       </c>
       <c r="K10" t="s">
         <v>12</v>
       </c>
       <c r="L10">
-        <v>506001</v>
+        <v>506367</v>
       </c>
     </row>
     <row r="11" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A11">
-        <v>9951407063</v>
+        <v>9390882143</v>
       </c>
       <c r="B11" t="s">
         <v>41</v>
       </c>
       <c r="C11">
-        <v>516</v>
+        <v>250</v>
       </c>
       <c r="D11" t="s">
         <v>10</v>
       </c>
       <c r="G11">
-        <v>2766</v>
+        <v>2802</v>
       </c>
       <c r="H11">
-        <v>46153</v>
+        <v>46166</v>
       </c>
       <c r="I11" t="s">
         <v>42</v>
       </c>
       <c r="J11" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="K11" t="s">
         <v>12</v>
       </c>
       <c r="L11">
-        <v>506370</v>
+        <v>506002</v>
       </c>
     </row>
     <row r="12" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A12">
-        <v>6364049832</v>
+        <v>9396387367</v>
       </c>
       <c r="B12" t="s">
         <v>43</v>
       </c>
       <c r="C12">
-        <v>501</v>
+        <v>2500</v>
       </c>
       <c r="D12" t="s">
         <v>10</v>
       </c>
       <c r="G12">
-        <v>2765</v>
+        <v>2800</v>
       </c>
       <c r="H12">
-        <v>46153</v>
+        <v>46166</v>
       </c>
       <c r="I12" t="s">
-        <v>24</v>
+        <v>44</v>
       </c>
       <c r="J12" t="s">
-        <v>24</v>
+        <v>13</v>
       </c>
       <c r="K12" t="s">
-        <v>25</v>
+        <v>12</v>
+      </c>
+      <c r="L12">
+        <v>506001</v>
       </c>
     </row>
     <row r="13" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A13">
-        <v>9866568921</v>
+        <v>9381179806</v>
       </c>
       <c r="B13" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="C13">
-        <v>2116</v>
+        <v>516</v>
       </c>
       <c r="D13" t="s">
         <v>10</v>
       </c>
       <c r="G13">
-        <v>2772</v>
+        <v>2809</v>
       </c>
       <c r="H13">
-        <v>46155</v>
+        <v>46169</v>
       </c>
       <c r="I13" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="J13" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="K13" t="s">
         <v>12</v>
       </c>
       <c r="L13">
-        <v>506002</v>
+        <v>506001</v>
       </c>
     </row>
     <row r="14" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A14">
-        <v>9959861405</v>
+        <v>8332969291</v>
       </c>
       <c r="B14" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="C14">
-        <v>1000</v>
+        <v>516</v>
       </c>
       <c r="D14" t="s">
         <v>10</v>
       </c>
       <c r="G14">
-        <v>2774</v>
+        <v>2818</v>
       </c>
       <c r="H14">
-        <v>46156</v>
+        <v>46170</v>
       </c>
       <c r="I14" t="s">
-        <v>47</v>
+        <v>48</v>
+      </c>
+      <c r="J14" t="s">
+        <v>11</v>
       </c>
       <c r="K14" t="s">
         <v>12</v>
       </c>
       <c r="L14">
-        <v>506002</v>
+        <v>506004</v>
       </c>
     </row>
     <row r="15" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A15">
-        <v>9494843093</v>
+        <v>9550803036</v>
       </c>
       <c r="B15" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="C15">
-        <v>2116</v>
+        <v>500</v>
       </c>
       <c r="D15" t="s">
         <v>10</v>
       </c>
       <c r="G15">
-        <v>2775</v>
+        <v>2817</v>
       </c>
       <c r="H15">
-        <v>46156</v>
+        <v>46170</v>
       </c>
       <c r="I15" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="J15" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="K15" t="s">
         <v>12</v>
       </c>
       <c r="L15">
-        <v>506001</v>
+        <v>506004</v>
       </c>
     </row>
     <row r="16" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A16">
-        <v>9963557727</v>
+        <v>8309890672</v>
       </c>
       <c r="B16" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="C16">
-        <v>501</v>
+        <v>500</v>
       </c>
       <c r="D16" t="s">
         <v>10</v>
       </c>
       <c r="G16">
-        <v>2776</v>
+        <v>2821</v>
       </c>
       <c r="H16">
-        <v>46156</v>
+        <v>46171</v>
       </c>
       <c r="I16" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="J16" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="K16" t="s">
         <v>12</v>
       </c>
       <c r="L16">
-        <v>506001</v>
+        <v>506006</v>
       </c>
     </row>
     <row r="17" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A17">
-        <v>7013220720</v>
+        <v>7674872512</v>
       </c>
       <c r="B17" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="C17">
-        <v>316</v>
+        <v>4000</v>
       </c>
       <c r="D17" t="s">
         <v>10</v>
       </c>
       <c r="G17">
-        <v>2777</v>
+        <v>2851</v>
       </c>
       <c r="H17">
-        <v>46157</v>
+        <v>46173</v>
       </c>
       <c r="I17" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="J17" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="K17" t="s">
         <v>12</v>
       </c>
       <c r="L17">
-        <v>506002</v>
+        <v>506001</v>
       </c>
     </row>
     <row r="18" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A18">
-        <v>7997093302</v>
+        <v>8106246466</v>
       </c>
       <c r="B18" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="C18">
-        <v>520</v>
+        <v>516</v>
       </c>
       <c r="D18" t="s">
         <v>10</v>
       </c>
       <c r="G18">
-        <v>2783</v>
+        <v>2831</v>
       </c>
       <c r="H18">
-        <v>46158</v>
+        <v>46174</v>
       </c>
       <c r="I18" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="J18" t="s">
         <v>11</v>
@@ -1546,65 +1465,65 @@
         <v>12</v>
       </c>
       <c r="L18">
-        <v>506142</v>
+        <v>506002</v>
       </c>
     </row>
     <row r="19" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A19">
-        <v>9704476844</v>
+        <v>9666334023</v>
       </c>
       <c r="B19" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="C19">
-        <v>520</v>
+        <v>516</v>
       </c>
       <c r="D19" t="s">
         <v>10</v>
       </c>
       <c r="G19">
-        <v>2782</v>
+        <v>2832</v>
       </c>
       <c r="H19">
-        <v>46158</v>
+        <v>46175</v>
       </c>
       <c r="I19" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="J19" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="K19" t="s">
         <v>12</v>
       </c>
       <c r="L19">
-        <v>506002</v>
+        <v>500092</v>
       </c>
     </row>
     <row r="20" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A20">
-        <v>9849502601</v>
+        <v>7732063430</v>
       </c>
       <c r="B20" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="C20">
-        <v>501</v>
+        <v>516</v>
       </c>
       <c r="D20" t="s">
         <v>10</v>
       </c>
       <c r="G20">
-        <v>2789</v>
+        <v>2833</v>
       </c>
       <c r="H20">
-        <v>46159</v>
+        <v>46175</v>
       </c>
       <c r="I20" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="J20" t="s">
-        <v>18</v>
+        <v>13</v>
       </c>
       <c r="K20" t="s">
         <v>12</v>
@@ -1615,57 +1534,57 @@
     </row>
     <row r="21" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A21">
-        <v>9959715373</v>
+        <v>8179583476</v>
       </c>
       <c r="B21" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="C21">
-        <v>520</v>
+        <v>516</v>
       </c>
       <c r="D21" t="s">
         <v>10</v>
       </c>
       <c r="G21">
-        <v>2781</v>
+        <v>2837</v>
       </c>
       <c r="H21">
-        <v>46160</v>
+        <v>46177</v>
       </c>
       <c r="I21" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="J21" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="K21" t="s">
         <v>12</v>
       </c>
       <c r="L21">
-        <v>506002</v>
+        <v>506001</v>
       </c>
     </row>
     <row r="22" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A22">
-        <v>9492781734</v>
+        <v>9390101462</v>
       </c>
       <c r="B22" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="C22">
-        <v>501</v>
+        <v>516</v>
       </c>
       <c r="D22" t="s">
         <v>10</v>
       </c>
       <c r="G22">
-        <v>2790</v>
+        <v>2838</v>
       </c>
       <c r="H22">
-        <v>46160</v>
+        <v>46177</v>
       </c>
       <c r="I22" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="J22" t="s">
         <v>13</v>
@@ -1679,57 +1598,57 @@
     </row>
     <row r="23" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A23">
-        <v>9705036449</v>
+        <v>6304730300</v>
       </c>
       <c r="B23" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="C23">
-        <v>500</v>
+        <v>516</v>
       </c>
       <c r="D23" t="s">
         <v>10</v>
       </c>
       <c r="G23">
-        <v>2793</v>
+        <v>2840</v>
       </c>
       <c r="H23">
-        <v>46163</v>
+        <v>46178</v>
       </c>
       <c r="I23" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="J23" t="s">
-        <v>19</v>
+        <v>11</v>
       </c>
       <c r="K23" t="s">
         <v>12</v>
       </c>
       <c r="L23">
-        <v>506169</v>
+        <v>506002</v>
       </c>
     </row>
     <row r="24" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A24">
-        <v>9030936319</v>
+        <v>9908900558</v>
       </c>
       <c r="B24" t="s">
-        <v>66</v>
+        <v>21</v>
       </c>
       <c r="C24">
-        <v>516</v>
+        <v>1011</v>
       </c>
       <c r="D24" t="s">
         <v>10</v>
       </c>
       <c r="G24">
-        <v>2794</v>
+        <v>2844</v>
       </c>
       <c r="H24">
-        <v>46164</v>
+        <v>46180</v>
       </c>
       <c r="I24" t="s">
-        <v>67</v>
+        <v>22</v>
       </c>
       <c r="J24" t="s">
         <v>13</v>
@@ -1743,153 +1662,153 @@
     </row>
     <row r="25" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A25">
-        <v>8985635919</v>
+        <v>8978506070</v>
       </c>
       <c r="B25" t="s">
+        <v>67</v>
+      </c>
+      <c r="C25">
+        <v>10016</v>
+      </c>
+      <c r="D25" t="s">
+        <v>10</v>
+      </c>
+      <c r="G25">
+        <v>2845</v>
+      </c>
+      <c r="H25">
+        <v>46180</v>
+      </c>
+      <c r="I25" t="s">
         <v>68</v>
       </c>
-      <c r="C25">
-        <v>520</v>
-      </c>
-      <c r="D25" t="s">
-        <v>10</v>
-      </c>
-      <c r="G25">
-        <v>2795</v>
-      </c>
-      <c r="H25">
-        <v>46165</v>
-      </c>
-      <c r="I25" t="s">
-        <v>69</v>
-      </c>
       <c r="J25" t="s">
-        <v>20</v>
+        <v>13</v>
       </c>
       <c r="K25" t="s">
         <v>12</v>
       </c>
       <c r="L25">
-        <v>506344</v>
+        <v>506001</v>
       </c>
     </row>
     <row r="26" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A26">
-        <v>8328376765</v>
+        <v>9849405377</v>
       </c>
       <c r="B26" t="s">
-        <v>70</v>
+        <v>15</v>
       </c>
       <c r="C26">
-        <v>500</v>
+        <v>10000</v>
       </c>
       <c r="D26" t="s">
         <v>10</v>
       </c>
       <c r="G26">
-        <v>2803</v>
+        <v>2847</v>
       </c>
       <c r="H26">
-        <v>46166</v>
+        <v>46180</v>
       </c>
       <c r="I26" t="s">
-        <v>71</v>
+        <v>16</v>
       </c>
       <c r="J26" t="s">
-        <v>20</v>
+        <v>13</v>
       </c>
       <c r="K26" t="s">
         <v>12</v>
       </c>
       <c r="L26">
-        <v>506367</v>
+        <v>506001</v>
       </c>
     </row>
     <row r="27" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A27">
-        <v>9390882143</v>
+        <v>8885665131</v>
       </c>
       <c r="B27" t="s">
-        <v>72</v>
+        <v>69</v>
       </c>
       <c r="C27">
-        <v>250</v>
+        <v>1116</v>
       </c>
       <c r="D27" t="s">
         <v>10</v>
       </c>
       <c r="G27">
-        <v>2802</v>
+        <v>2856</v>
       </c>
       <c r="H27">
-        <v>46166</v>
+        <v>46182</v>
       </c>
       <c r="I27" t="s">
-        <v>73</v>
+        <v>70</v>
       </c>
       <c r="J27" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="K27" t="s">
         <v>12</v>
       </c>
       <c r="L27">
-        <v>506002</v>
+        <v>506003</v>
       </c>
     </row>
     <row r="28" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A28">
-        <v>9396387367</v>
+        <v>9618551013</v>
       </c>
       <c r="B28" t="s">
-        <v>74</v>
+        <v>71</v>
       </c>
       <c r="C28">
-        <v>2500</v>
+        <v>5000</v>
       </c>
       <c r="D28" t="s">
         <v>10</v>
       </c>
       <c r="G28">
-        <v>2800</v>
+        <v>2857</v>
       </c>
       <c r="H28">
-        <v>46166</v>
+        <v>46182</v>
       </c>
       <c r="I28" t="s">
-        <v>75</v>
+        <v>72</v>
       </c>
       <c r="J28" t="s">
-        <v>13</v>
+        <v>73</v>
       </c>
       <c r="K28" t="s">
         <v>12</v>
       </c>
       <c r="L28">
-        <v>506001</v>
+        <v>507302</v>
       </c>
     </row>
     <row r="29" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A29">
-        <v>9381179806</v>
+        <v>9573818089</v>
       </c>
       <c r="B29" t="s">
-        <v>76</v>
+        <v>74</v>
       </c>
       <c r="C29">
-        <v>516</v>
+        <v>2116</v>
       </c>
       <c r="D29" t="s">
         <v>10</v>
       </c>
       <c r="G29">
-        <v>2809</v>
+        <v>2861</v>
       </c>
       <c r="H29">
-        <v>46169</v>
+        <v>46184</v>
       </c>
       <c r="I29" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="J29" t="s">
         <v>13</v>
@@ -1903,10 +1822,10 @@
     </row>
     <row r="30" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A30">
-        <v>8332969291</v>
+        <v>9440048427</v>
       </c>
       <c r="B30" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
       <c r="C30">
         <v>516</v>
@@ -1915,141 +1834,141 @@
         <v>10</v>
       </c>
       <c r="G30">
-        <v>2818</v>
+        <v>2860</v>
       </c>
       <c r="H30">
-        <v>46170</v>
+        <v>46184</v>
       </c>
       <c r="I30" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="J30" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="K30" t="s">
         <v>12</v>
       </c>
       <c r="L30">
-        <v>506004</v>
+        <v>506009</v>
       </c>
     </row>
     <row r="31" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A31">
-        <v>9550803036</v>
+        <v>9885809376</v>
       </c>
       <c r="B31" t="s">
+        <v>78</v>
+      </c>
+      <c r="C31">
+        <v>501</v>
+      </c>
+      <c r="D31" t="s">
+        <v>10</v>
+      </c>
+      <c r="G31">
+        <v>2862</v>
+      </c>
+      <c r="H31">
+        <v>46184</v>
+      </c>
+      <c r="I31" t="s">
+        <v>79</v>
+      </c>
+      <c r="J31" t="s">
         <v>80</v>
       </c>
-      <c r="C31">
-        <v>500</v>
-      </c>
-      <c r="D31" t="s">
-        <v>10</v>
-      </c>
-      <c r="G31">
-        <v>2817</v>
-      </c>
-      <c r="H31">
-        <v>46170</v>
-      </c>
-      <c r="I31" t="s">
-        <v>81</v>
-      </c>
-      <c r="J31" t="s">
-        <v>11</v>
-      </c>
       <c r="K31" t="s">
         <v>12</v>
       </c>
       <c r="L31">
-        <v>506004</v>
+        <v>500090</v>
       </c>
     </row>
     <row r="32" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A32">
-        <v>8309890672</v>
+        <v>8919698473</v>
       </c>
       <c r="B32" t="s">
+        <v>81</v>
+      </c>
+      <c r="C32">
+        <v>1200</v>
+      </c>
+      <c r="D32" t="s">
+        <v>10</v>
+      </c>
+      <c r="G32">
+        <v>2867</v>
+      </c>
+      <c r="H32">
+        <v>46185</v>
+      </c>
+      <c r="I32" t="s">
         <v>82</v>
       </c>
-      <c r="C32">
-        <v>500</v>
-      </c>
-      <c r="D32" t="s">
-        <v>10</v>
-      </c>
-      <c r="G32">
-        <v>2821</v>
-      </c>
-      <c r="H32">
-        <v>46171</v>
-      </c>
-      <c r="I32" t="s">
-        <v>83</v>
-      </c>
       <c r="J32" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="K32" t="s">
         <v>12</v>
       </c>
       <c r="L32">
-        <v>506006</v>
+        <v>506001</v>
       </c>
     </row>
     <row r="33" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A33">
-        <v>7674872512</v>
+        <v>9989283504</v>
       </c>
       <c r="B33" t="s">
+        <v>83</v>
+      </c>
+      <c r="C33">
+        <v>520</v>
+      </c>
+      <c r="D33" t="s">
+        <v>10</v>
+      </c>
+      <c r="G33">
+        <v>2870</v>
+      </c>
+      <c r="H33">
+        <v>46185</v>
+      </c>
+      <c r="I33" t="s">
         <v>84</v>
       </c>
-      <c r="C33">
-        <v>4000</v>
-      </c>
-      <c r="D33" t="s">
-        <v>10</v>
-      </c>
-      <c r="G33">
-        <v>2851</v>
-      </c>
-      <c r="H33">
-        <v>46173</v>
-      </c>
-      <c r="I33" t="s">
-        <v>85</v>
-      </c>
       <c r="J33" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="K33" t="s">
         <v>12</v>
       </c>
       <c r="L33">
-        <v>506001</v>
+        <v>506356</v>
       </c>
     </row>
     <row r="34" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A34">
-        <v>8106246466</v>
+        <v>9160327916</v>
       </c>
       <c r="B34" t="s">
+        <v>85</v>
+      </c>
+      <c r="C34">
+        <v>520</v>
+      </c>
+      <c r="D34" t="s">
+        <v>10</v>
+      </c>
+      <c r="G34">
+        <v>2873</v>
+      </c>
+      <c r="H34">
+        <v>46186</v>
+      </c>
+      <c r="I34" t="s">
         <v>86</v>
-      </c>
-      <c r="C34">
-        <v>516</v>
-      </c>
-      <c r="D34" t="s">
-        <v>10</v>
-      </c>
-      <c r="G34">
-        <v>2831</v>
-      </c>
-      <c r="H34">
-        <v>46174</v>
-      </c>
-      <c r="I34" t="s">
-        <v>87</v>
       </c>
       <c r="J34" t="s">
         <v>11</v>
@@ -2058,62 +1977,62 @@
         <v>12</v>
       </c>
       <c r="L34">
-        <v>506002</v>
+        <v>506122</v>
       </c>
     </row>
     <row r="35" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A35">
-        <v>9666334023</v>
+        <v>9440983869</v>
       </c>
       <c r="B35" t="s">
+        <v>87</v>
+      </c>
+      <c r="C35">
+        <v>1000</v>
+      </c>
+      <c r="D35" t="s">
+        <v>10</v>
+      </c>
+      <c r="G35">
+        <v>2251</v>
+      </c>
+      <c r="H35">
+        <v>46186</v>
+      </c>
+      <c r="I35" t="s">
         <v>88</v>
       </c>
-      <c r="C35">
-        <v>516</v>
-      </c>
-      <c r="D35" t="s">
-        <v>10</v>
-      </c>
-      <c r="G35">
-        <v>2832</v>
-      </c>
-      <c r="H35">
-        <v>46175</v>
-      </c>
-      <c r="I35" t="s">
+      <c r="J35" t="s">
         <v>89</v>
       </c>
-      <c r="J35" t="s">
-        <v>13</v>
-      </c>
       <c r="K35" t="s">
-        <v>12</v>
+        <v>90</v>
       </c>
       <c r="L35">
-        <v>500092</v>
+        <v>327022</v>
       </c>
     </row>
     <row r="36" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A36">
-        <v>7732063430</v>
+        <v>9177357957</v>
       </c>
       <c r="B36" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="C36">
-        <v>516</v>
+        <v>500</v>
       </c>
       <c r="D36" t="s">
         <v>10</v>
       </c>
       <c r="G36">
-        <v>2833</v>
+        <v>2886</v>
       </c>
       <c r="H36">
-        <v>46175</v>
+        <v>46187</v>
       </c>
       <c r="I36" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="J36" t="s">
         <v>13</v>
@@ -2122,33 +2041,33 @@
         <v>12</v>
       </c>
       <c r="L36">
-        <v>506003</v>
+        <v>506001</v>
       </c>
     </row>
     <row r="37" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A37">
-        <v>8179583476</v>
+        <v>9963437378</v>
       </c>
       <c r="B37" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="C37">
-        <v>516</v>
+        <v>1500</v>
       </c>
       <c r="D37" t="s">
         <v>10</v>
       </c>
       <c r="G37">
-        <v>2837</v>
+        <v>2881</v>
       </c>
       <c r="H37">
-        <v>46177</v>
+        <v>46187</v>
       </c>
       <c r="I37" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="J37" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="K37" t="s">
         <v>12</v>
@@ -2159,22 +2078,22 @@
     </row>
     <row r="38" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A38">
-        <v>9390101462</v>
+        <v>9963437378</v>
       </c>
       <c r="B38" t="s">
-        <v>94</v>
+        <v>17</v>
       </c>
       <c r="C38">
-        <v>516</v>
+        <v>520</v>
       </c>
       <c r="D38" t="s">
         <v>10</v>
       </c>
       <c r="G38">
-        <v>2838</v>
+        <v>2877</v>
       </c>
       <c r="H38">
-        <v>46177</v>
+        <v>46187</v>
       </c>
       <c r="I38" t="s">
         <v>95</v>
@@ -2191,249 +2110,237 @@
     </row>
     <row r="39" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A39">
-        <v>6304730300</v>
+        <v>9000235756</v>
       </c>
       <c r="B39" t="s">
         <v>96</v>
       </c>
       <c r="C39">
-        <v>516</v>
+        <v>616</v>
       </c>
       <c r="D39" t="s">
         <v>10</v>
       </c>
       <c r="G39">
-        <v>2840</v>
+        <v>2888</v>
       </c>
       <c r="H39">
-        <v>46178</v>
+        <v>46187</v>
       </c>
       <c r="I39" t="s">
         <v>97</v>
       </c>
       <c r="J39" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="K39" t="s">
         <v>12</v>
       </c>
       <c r="L39">
-        <v>506002</v>
+        <v>506001</v>
       </c>
     </row>
     <row r="40" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A40">
-        <v>9908900558</v>
+        <v>7382447229</v>
       </c>
       <c r="B40" t="s">
-        <v>21</v>
+        <v>98</v>
       </c>
       <c r="C40">
-        <v>1011</v>
+        <v>25116</v>
       </c>
       <c r="D40" t="s">
         <v>10</v>
       </c>
       <c r="G40">
-        <v>2844</v>
+        <v>2885</v>
       </c>
       <c r="H40">
-        <v>46180</v>
+        <v>46187</v>
       </c>
       <c r="I40" t="s">
-        <v>22</v>
-      </c>
-      <c r="J40" t="s">
-        <v>13</v>
+        <v>99</v>
       </c>
       <c r="K40" t="s">
         <v>12</v>
-      </c>
-      <c r="L40">
-        <v>506001</v>
       </c>
     </row>
     <row r="41" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A41">
-        <v>8978506070</v>
+        <v>7780370611</v>
       </c>
       <c r="B41" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="C41">
-        <v>10016</v>
+        <v>516</v>
       </c>
       <c r="D41" t="s">
         <v>10</v>
       </c>
       <c r="G41">
-        <v>2845</v>
+        <v>2893</v>
       </c>
       <c r="H41">
-        <v>46180</v>
+        <v>46188</v>
       </c>
       <c r="I41" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="J41" t="s">
-        <v>13</v>
+        <v>102</v>
       </c>
       <c r="K41" t="s">
         <v>12</v>
       </c>
       <c r="L41">
-        <v>506001</v>
+        <v>502280</v>
       </c>
     </row>
     <row r="42" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A42">
-        <v>9849405377</v>
+        <v>9397398024</v>
       </c>
       <c r="B42" t="s">
-        <v>15</v>
+        <v>103</v>
       </c>
       <c r="C42">
-        <v>10000</v>
+        <v>2505</v>
       </c>
       <c r="D42" t="s">
         <v>10</v>
       </c>
       <c r="G42">
-        <v>2847</v>
+        <v>2895</v>
       </c>
       <c r="H42">
-        <v>46180</v>
+        <v>46189</v>
       </c>
       <c r="I42" t="s">
-        <v>16</v>
-      </c>
-      <c r="J42" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="K42" t="s">
         <v>12</v>
-      </c>
-      <c r="L42">
-        <v>506001</v>
       </c>
     </row>
     <row r="43" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A43">
-        <v>8885665131</v>
+        <v>8106576085</v>
       </c>
       <c r="B43" t="s">
-        <v>100</v>
+        <v>104</v>
       </c>
       <c r="C43">
-        <v>1116</v>
+        <v>520</v>
       </c>
       <c r="D43" t="s">
         <v>10</v>
       </c>
       <c r="G43">
-        <v>2856</v>
+        <v>2897</v>
       </c>
       <c r="H43">
-        <v>46182</v>
+        <v>46190</v>
       </c>
       <c r="I43" t="s">
-        <v>101</v>
+        <v>105</v>
       </c>
       <c r="J43" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="K43" t="s">
         <v>12</v>
       </c>
       <c r="L43">
-        <v>506003</v>
+        <v>506002</v>
       </c>
     </row>
     <row r="44" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A44">
-        <v>9618551013</v>
+        <v>7993717797</v>
       </c>
       <c r="B44" t="s">
-        <v>102</v>
+        <v>106</v>
       </c>
       <c r="C44">
-        <v>5000</v>
+        <v>516</v>
       </c>
       <c r="D44" t="s">
         <v>10</v>
       </c>
       <c r="G44">
-        <v>2857</v>
+        <v>2898</v>
       </c>
       <c r="H44">
-        <v>46182</v>
+        <v>46190</v>
       </c>
       <c r="I44" t="s">
-        <v>103</v>
+        <v>107</v>
       </c>
       <c r="J44" t="s">
-        <v>104</v>
+        <v>13</v>
       </c>
       <c r="K44" t="s">
         <v>12</v>
       </c>
       <c r="L44">
-        <v>507302</v>
+        <v>506001</v>
       </c>
     </row>
     <row r="45" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A45">
-        <v>9573818089</v>
+        <v>9177177356</v>
       </c>
       <c r="B45" t="s">
-        <v>105</v>
+        <v>108</v>
       </c>
       <c r="C45">
-        <v>2116</v>
+        <v>500</v>
       </c>
       <c r="D45" t="s">
         <v>10</v>
       </c>
       <c r="G45">
-        <v>2861</v>
+        <v>2351</v>
       </c>
       <c r="H45">
-        <v>46184</v>
+        <v>46192</v>
       </c>
       <c r="I45" t="s">
-        <v>106</v>
+        <v>109</v>
       </c>
       <c r="J45" t="s">
-        <v>13</v>
+        <v>19</v>
       </c>
       <c r="K45" t="s">
         <v>12</v>
       </c>
       <c r="L45">
-        <v>506001</v>
+        <v>5060169</v>
       </c>
     </row>
     <row r="46" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A46">
-        <v>9440048427</v>
+        <v>9701817002</v>
       </c>
       <c r="B46" t="s">
-        <v>107</v>
+        <v>110</v>
       </c>
       <c r="C46">
-        <v>516</v>
+        <v>500</v>
       </c>
       <c r="D46" t="s">
         <v>10</v>
       </c>
       <c r="G46">
-        <v>2860</v>
+        <v>2352</v>
       </c>
       <c r="H46">
-        <v>46184</v>
+        <v>46192</v>
       </c>
       <c r="I46" t="s">
-        <v>108</v>
+        <v>111</v>
       </c>
       <c r="J46" t="s">
         <v>13</v>
@@ -2442,79 +2349,79 @@
         <v>12</v>
       </c>
       <c r="L46">
-        <v>506009</v>
+        <v>506001</v>
       </c>
     </row>
     <row r="47" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A47">
-        <v>9885809376</v>
+        <v>8500823588</v>
       </c>
       <c r="B47" t="s">
-        <v>109</v>
+        <v>112</v>
       </c>
       <c r="C47">
-        <v>501</v>
+        <v>5116</v>
       </c>
       <c r="D47" t="s">
         <v>10</v>
       </c>
       <c r="G47">
-        <v>2862</v>
+        <v>2900</v>
       </c>
       <c r="H47">
-        <v>46184</v>
+        <v>46192</v>
       </c>
       <c r="I47" t="s">
-        <v>110</v>
+        <v>113</v>
       </c>
       <c r="J47" t="s">
-        <v>111</v>
+        <v>13</v>
       </c>
       <c r="K47" t="s">
         <v>12</v>
       </c>
       <c r="L47">
-        <v>500090</v>
+        <v>506001</v>
       </c>
     </row>
     <row r="48" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A48">
-        <v>8919698473</v>
+        <v>8096496813</v>
       </c>
       <c r="B48" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="C48">
-        <v>1200</v>
+        <v>500</v>
       </c>
       <c r="D48" t="s">
         <v>10</v>
       </c>
       <c r="G48">
-        <v>2867</v>
+        <v>2356</v>
       </c>
       <c r="H48">
-        <v>46185</v>
+        <v>46193</v>
       </c>
       <c r="I48" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="J48" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="K48" t="s">
         <v>12</v>
       </c>
       <c r="L48">
-        <v>506001</v>
+        <v>506002</v>
       </c>
     </row>
     <row r="49" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A49">
-        <v>9989283504</v>
+        <v>9849562822</v>
       </c>
       <c r="B49" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="C49">
         <v>520</v>
@@ -2523,13 +2430,13 @@
         <v>10</v>
       </c>
       <c r="G49">
-        <v>2870</v>
+        <v>2362</v>
       </c>
       <c r="H49">
-        <v>46185</v>
+        <v>46195</v>
       </c>
       <c r="I49" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
       <c r="J49" t="s">
         <v>11</v>
@@ -2538,30 +2445,30 @@
         <v>12</v>
       </c>
       <c r="L49">
-        <v>506356</v>
+        <v>506002</v>
       </c>
     </row>
     <row r="50" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A50">
-        <v>9160327916</v>
+        <v>9782833030</v>
       </c>
       <c r="B50" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="C50">
-        <v>520</v>
+        <v>5100</v>
       </c>
       <c r="D50" t="s">
         <v>10</v>
       </c>
       <c r="G50">
-        <v>2873</v>
+        <v>2363</v>
       </c>
       <c r="H50">
-        <v>46186</v>
+        <v>46196</v>
       </c>
       <c r="I50" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="J50" t="s">
         <v>11</v>
@@ -2570,97 +2477,97 @@
         <v>12</v>
       </c>
       <c r="L50">
-        <v>506122</v>
+        <v>506002</v>
       </c>
     </row>
     <row r="51" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A51">
-        <v>9440983869</v>
+        <v>9907978092</v>
       </c>
       <c r="B51" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="C51">
-        <v>1000</v>
+        <v>500</v>
       </c>
       <c r="D51" t="s">
         <v>10</v>
       </c>
       <c r="G51">
-        <v>2251</v>
+        <v>2366</v>
       </c>
       <c r="H51">
-        <v>46186</v>
+        <v>46197</v>
       </c>
       <c r="I51" t="s">
-        <v>119</v>
+        <v>121</v>
       </c>
       <c r="J51" t="s">
-        <v>120</v>
+        <v>13</v>
       </c>
       <c r="K51" t="s">
-        <v>121</v>
+        <v>12</v>
       </c>
       <c r="L51">
-        <v>327022</v>
+        <v>506001</v>
       </c>
     </row>
     <row r="52" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A52">
-        <v>9177357957</v>
+        <v>9849944801</v>
       </c>
       <c r="B52" t="s">
         <v>122</v>
       </c>
       <c r="C52">
-        <v>500</v>
+        <v>1011</v>
       </c>
       <c r="D52" t="s">
         <v>10</v>
       </c>
       <c r="G52">
-        <v>2886</v>
+        <v>2370</v>
       </c>
       <c r="H52">
-        <v>46187</v>
+        <v>46198</v>
       </c>
       <c r="I52" t="s">
         <v>123</v>
       </c>
       <c r="J52" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="K52" t="s">
         <v>12</v>
       </c>
       <c r="L52">
-        <v>506001</v>
+        <v>506002</v>
       </c>
     </row>
     <row r="53" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A53">
-        <v>9963437378</v>
+        <v>9866217386</v>
       </c>
       <c r="B53" t="s">
         <v>124</v>
       </c>
       <c r="C53">
-        <v>1500</v>
+        <v>516</v>
       </c>
       <c r="D53" t="s">
         <v>10</v>
       </c>
       <c r="G53">
-        <v>2881</v>
+        <v>2367</v>
       </c>
       <c r="H53">
-        <v>46187</v>
+        <v>46198</v>
       </c>
       <c r="I53" t="s">
         <v>125</v>
       </c>
       <c r="J53" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="K53" t="s">
         <v>12</v>
@@ -2671,25 +2578,25 @@
     </row>
     <row r="54" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A54">
-        <v>9963437378</v>
+        <v>8686858643</v>
       </c>
       <c r="B54" t="s">
-        <v>17</v>
+        <v>126</v>
       </c>
       <c r="C54">
-        <v>520</v>
+        <v>500</v>
       </c>
       <c r="D54" t="s">
         <v>10</v>
       </c>
       <c r="G54">
-        <v>2877</v>
+        <v>2373</v>
       </c>
       <c r="H54">
-        <v>46187</v>
+        <v>46199</v>
       </c>
       <c r="I54" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="J54" t="s">
         <v>13</v>
@@ -2703,158 +2610,167 @@
     </row>
     <row r="55" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A55">
-        <v>9000235756</v>
+        <v>9848224298</v>
       </c>
       <c r="B55" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="C55">
-        <v>616</v>
+        <v>520</v>
       </c>
       <c r="D55" t="s">
         <v>10</v>
       </c>
       <c r="G55">
-        <v>2888</v>
+        <v>2374</v>
       </c>
       <c r="H55">
-        <v>46187</v>
+        <v>46199</v>
       </c>
       <c r="I55" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="J55" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="K55" t="s">
         <v>12</v>
       </c>
       <c r="L55">
-        <v>506001</v>
+        <v>5016164</v>
       </c>
     </row>
     <row r="56" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A56">
-        <v>7382447229</v>
+        <v>8885665131</v>
       </c>
       <c r="B56" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="C56">
-        <v>25116</v>
+        <v>100116</v>
       </c>
       <c r="D56" t="s">
         <v>10</v>
       </c>
       <c r="G56">
-        <v>2885</v>
+        <v>2375</v>
       </c>
       <c r="H56">
-        <v>46187</v>
+        <v>46199</v>
       </c>
       <c r="I56" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="K56" t="s">
         <v>12</v>
+      </c>
+      <c r="L56">
+        <v>506003</v>
       </c>
     </row>
     <row r="57" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A57">
-        <v>7780370611</v>
+        <v>8466927579</v>
       </c>
       <c r="B57" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="C57">
-        <v>516</v>
+        <v>520</v>
       </c>
       <c r="D57" t="s">
         <v>10</v>
       </c>
       <c r="G57">
-        <v>2893</v>
+        <v>2376</v>
       </c>
       <c r="H57">
-        <v>46188</v>
+        <v>46200</v>
       </c>
       <c r="I57" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="J57" t="s">
-        <v>133</v>
+        <v>11</v>
       </c>
       <c r="K57" t="s">
         <v>12</v>
       </c>
       <c r="L57">
-        <v>502280</v>
+        <v>506005</v>
       </c>
     </row>
     <row r="58" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A58">
-        <v>9397398024</v>
+        <v>9603557182</v>
       </c>
       <c r="B58" t="s">
         <v>134</v>
       </c>
       <c r="C58">
-        <v>2505</v>
+        <v>516</v>
       </c>
       <c r="D58" t="s">
         <v>10</v>
       </c>
       <c r="G58">
-        <v>2895</v>
+        <v>2378</v>
       </c>
       <c r="H58">
-        <v>46189</v>
+        <v>46201</v>
       </c>
       <c r="I58" t="s">
-        <v>14</v>
+        <v>135</v>
+      </c>
+      <c r="J58" t="s">
+        <v>13</v>
       </c>
       <c r="K58" t="s">
         <v>12</v>
+      </c>
+      <c r="L58">
+        <v>505101</v>
       </c>
     </row>
     <row r="59" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A59">
-        <v>8106576085</v>
+        <v>9490100604</v>
       </c>
       <c r="B59" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="C59">
-        <v>520</v>
+        <v>1116</v>
       </c>
       <c r="D59" t="s">
         <v>10</v>
       </c>
       <c r="G59">
-        <v>2897</v>
+        <v>2377</v>
       </c>
       <c r="H59">
-        <v>46190</v>
+        <v>46201</v>
       </c>
       <c r="I59" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="J59" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="K59" t="s">
         <v>12</v>
       </c>
       <c r="L59">
-        <v>506002</v>
+        <v>506001</v>
       </c>
     </row>
     <row r="60" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A60">
-        <v>7993717797</v>
+        <v>9542895197</v>
       </c>
       <c r="B60" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="C60">
         <v>516</v>
@@ -2863,77 +2779,77 @@
         <v>10</v>
       </c>
       <c r="G60">
-        <v>2898</v>
+        <v>2379</v>
       </c>
       <c r="H60">
-        <v>46190</v>
+        <v>46201</v>
       </c>
       <c r="I60" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="J60" t="s">
-        <v>13</v>
+        <v>140</v>
       </c>
       <c r="K60" t="s">
         <v>12</v>
       </c>
       <c r="L60">
-        <v>506001</v>
+        <v>502103</v>
       </c>
     </row>
     <row r="61" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A61">
-        <v>9177177356</v>
+        <v>7893800980</v>
       </c>
       <c r="B61" t="s">
-        <v>139</v>
+        <v>141</v>
       </c>
       <c r="C61">
-        <v>500</v>
+        <v>520</v>
       </c>
       <c r="D61" t="s">
         <v>10</v>
       </c>
       <c r="G61">
-        <v>2351</v>
+        <v>2380</v>
       </c>
       <c r="H61">
-        <v>46192</v>
+        <v>46201</v>
       </c>
       <c r="I61" t="s">
-        <v>140</v>
+        <v>142</v>
       </c>
       <c r="J61" t="s">
-        <v>19</v>
+        <v>11</v>
       </c>
       <c r="K61" t="s">
         <v>12</v>
       </c>
       <c r="L61">
-        <v>5060169</v>
+        <v>506002</v>
       </c>
     </row>
     <row r="62" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A62">
-        <v>9701817002</v>
+        <v>9849212083</v>
       </c>
       <c r="B62" t="s">
-        <v>141</v>
+        <v>143</v>
       </c>
       <c r="C62">
-        <v>500</v>
+        <v>3201</v>
       </c>
       <c r="D62" t="s">
         <v>10</v>
       </c>
       <c r="G62">
-        <v>2352</v>
+        <v>2388</v>
       </c>
       <c r="H62">
-        <v>46192</v>
+        <v>46202</v>
       </c>
       <c r="I62" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="J62" t="s">
         <v>13</v>
@@ -2947,25 +2863,25 @@
     </row>
     <row r="63" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A63">
-        <v>8500823588</v>
+        <v>8500288366</v>
       </c>
       <c r="B63" t="s">
-        <v>143</v>
+        <v>145</v>
       </c>
       <c r="C63">
-        <v>5116</v>
+        <v>516</v>
       </c>
       <c r="D63" t="s">
         <v>10</v>
       </c>
       <c r="G63">
-        <v>2900</v>
+        <v>2389</v>
       </c>
       <c r="H63">
-        <v>46192</v>
+        <v>46202</v>
       </c>
       <c r="I63" t="s">
-        <v>144</v>
+        <v>146</v>
       </c>
       <c r="J63" t="s">
         <v>13</v>
@@ -2979,57 +2895,57 @@
     </row>
     <row r="64" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A64">
-        <v>8096496813</v>
+        <v>8500288366</v>
       </c>
       <c r="B64" t="s">
-        <v>145</v>
+        <v>147</v>
       </c>
       <c r="C64">
-        <v>500</v>
+        <v>1116</v>
       </c>
       <c r="D64" t="s">
         <v>10</v>
       </c>
       <c r="G64">
-        <v>2356</v>
+        <v>2387</v>
       </c>
       <c r="H64">
-        <v>46193</v>
+        <v>46202</v>
       </c>
       <c r="I64" t="s">
-        <v>146</v>
+        <v>148</v>
       </c>
       <c r="J64" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="K64" t="s">
         <v>12</v>
       </c>
       <c r="L64">
-        <v>506002</v>
+        <v>506001</v>
       </c>
     </row>
     <row r="65" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A65">
-        <v>9849562822</v>
+        <v>9032375368</v>
       </c>
       <c r="B65" t="s">
-        <v>147</v>
+        <v>149</v>
       </c>
       <c r="C65">
-        <v>520</v>
+        <v>516</v>
       </c>
       <c r="D65" t="s">
         <v>10</v>
       </c>
       <c r="G65">
-        <v>2362</v>
+        <v>2386</v>
       </c>
       <c r="H65">
-        <v>46195</v>
+        <v>46202</v>
       </c>
       <c r="I65" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="J65" t="s">
         <v>11</v>
@@ -3038,611 +2954,102 @@
         <v>12</v>
       </c>
       <c r="L65">
-        <v>506002</v>
+        <v>506003</v>
       </c>
     </row>
     <row r="66" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A66">
-        <v>9782833030</v>
+        <v>9908900558</v>
       </c>
       <c r="B66" t="s">
-        <v>149</v>
+        <v>21</v>
       </c>
       <c r="C66">
-        <v>5100</v>
+        <v>51000</v>
       </c>
       <c r="D66" t="s">
         <v>10</v>
       </c>
       <c r="G66">
-        <v>2363</v>
+        <v>2385</v>
       </c>
       <c r="H66">
-        <v>46196</v>
+        <v>46202</v>
       </c>
       <c r="I66" t="s">
-        <v>150</v>
+        <v>22</v>
       </c>
       <c r="J66" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="K66" t="s">
         <v>12</v>
       </c>
       <c r="L66">
-        <v>506002</v>
+        <v>506001</v>
       </c>
     </row>
     <row r="67" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A67">
-        <v>9907978092</v>
+        <v>9866568921</v>
       </c>
       <c r="B67" t="s">
         <v>151</v>
       </c>
       <c r="C67">
-        <v>500</v>
+        <v>501</v>
       </c>
       <c r="D67" t="s">
         <v>10</v>
       </c>
       <c r="G67">
-        <v>2366</v>
+        <v>2392</v>
       </c>
       <c r="H67">
-        <v>46197</v>
+        <v>46202</v>
       </c>
       <c r="I67" t="s">
         <v>152</v>
       </c>
       <c r="J67" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="K67" t="s">
         <v>12</v>
       </c>
       <c r="L67">
-        <v>506001</v>
+        <v>506002</v>
       </c>
     </row>
     <row r="68" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A68">
-        <v>9849944801</v>
+        <v>9652525448</v>
       </c>
       <c r="B68" t="s">
         <v>153</v>
       </c>
       <c r="C68">
-        <v>1011</v>
+        <v>516</v>
       </c>
       <c r="D68" t="s">
         <v>10</v>
       </c>
       <c r="G68">
-        <v>2370</v>
+        <v>2393</v>
       </c>
       <c r="H68">
-        <v>46198</v>
+        <v>46203</v>
       </c>
       <c r="I68" t="s">
         <v>154</v>
       </c>
       <c r="J68" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="K68" t="s">
         <v>12</v>
       </c>
       <c r="L68">
-        <v>506002</v>
-      </c>
-    </row>
-    <row r="69" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A69">
-        <v>9866217386</v>
-      </c>
-      <c r="B69" t="s">
-        <v>155</v>
-      </c>
-      <c r="C69">
-        <v>516</v>
-      </c>
-      <c r="D69" t="s">
-        <v>10</v>
-      </c>
-      <c r="G69">
-        <v>2367</v>
-      </c>
-      <c r="H69">
-        <v>46198</v>
-      </c>
-      <c r="I69" t="s">
-        <v>156</v>
-      </c>
-      <c r="J69" t="s">
-        <v>13</v>
-      </c>
-      <c r="K69" t="s">
-        <v>12</v>
-      </c>
-      <c r="L69">
-        <v>506001</v>
-      </c>
-    </row>
-    <row r="70" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A70">
-        <v>8686858643</v>
-      </c>
-      <c r="B70" t="s">
-        <v>157</v>
-      </c>
-      <c r="C70">
-        <v>500</v>
-      </c>
-      <c r="D70" t="s">
-        <v>10</v>
-      </c>
-      <c r="G70">
-        <v>2373</v>
-      </c>
-      <c r="H70">
-        <v>46199</v>
-      </c>
-      <c r="I70" t="s">
-        <v>158</v>
-      </c>
-      <c r="J70" t="s">
-        <v>13</v>
-      </c>
-      <c r="K70" t="s">
-        <v>12</v>
-      </c>
-      <c r="L70">
-        <v>506001</v>
-      </c>
-    </row>
-    <row r="71" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A71">
-        <v>9848224298</v>
-      </c>
-      <c r="B71" t="s">
-        <v>159</v>
-      </c>
-      <c r="C71">
-        <v>520</v>
-      </c>
-      <c r="D71" t="s">
-        <v>10</v>
-      </c>
-      <c r="G71">
-        <v>2374</v>
-      </c>
-      <c r="H71">
-        <v>46199</v>
-      </c>
-      <c r="I71" t="s">
-        <v>160</v>
-      </c>
-      <c r="J71" t="s">
-        <v>11</v>
-      </c>
-      <c r="K71" t="s">
-        <v>12</v>
-      </c>
-      <c r="L71">
-        <v>5016164</v>
-      </c>
-    </row>
-    <row r="72" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A72">
-        <v>8885665131</v>
-      </c>
-      <c r="B72" t="s">
-        <v>161</v>
-      </c>
-      <c r="C72">
-        <v>100116</v>
-      </c>
-      <c r="D72" t="s">
-        <v>10</v>
-      </c>
-      <c r="G72">
-        <v>2375</v>
-      </c>
-      <c r="H72">
-        <v>46199</v>
-      </c>
-      <c r="I72" t="s">
-        <v>162</v>
-      </c>
-      <c r="K72" t="s">
-        <v>12</v>
-      </c>
-      <c r="L72">
-        <v>506003</v>
-      </c>
-    </row>
-    <row r="73" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A73">
-        <v>8466927579</v>
-      </c>
-      <c r="B73" t="s">
-        <v>163</v>
-      </c>
-      <c r="C73">
-        <v>520</v>
-      </c>
-      <c r="D73" t="s">
-        <v>10</v>
-      </c>
-      <c r="G73">
-        <v>2376</v>
-      </c>
-      <c r="H73">
-        <v>46200</v>
-      </c>
-      <c r="I73" t="s">
-        <v>164</v>
-      </c>
-      <c r="J73" t="s">
-        <v>11</v>
-      </c>
-      <c r="K73" t="s">
-        <v>12</v>
-      </c>
-      <c r="L73">
-        <v>506005</v>
-      </c>
-    </row>
-    <row r="74" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A74">
-        <v>9603557182</v>
-      </c>
-      <c r="B74" t="s">
-        <v>165</v>
-      </c>
-      <c r="C74">
-        <v>516</v>
-      </c>
-      <c r="D74" t="s">
-        <v>10</v>
-      </c>
-      <c r="G74">
-        <v>2378</v>
-      </c>
-      <c r="H74">
-        <v>46201</v>
-      </c>
-      <c r="I74" t="s">
-        <v>166</v>
-      </c>
-      <c r="J74" t="s">
-        <v>13</v>
-      </c>
-      <c r="K74" t="s">
-        <v>12</v>
-      </c>
-      <c r="L74">
-        <v>505101</v>
-      </c>
-    </row>
-    <row r="75" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A75">
-        <v>9490100604</v>
-      </c>
-      <c r="B75" t="s">
-        <v>167</v>
-      </c>
-      <c r="C75">
-        <v>1116</v>
-      </c>
-      <c r="D75" t="s">
-        <v>10</v>
-      </c>
-      <c r="G75">
-        <v>2377</v>
-      </c>
-      <c r="H75">
-        <v>46201</v>
-      </c>
-      <c r="I75" t="s">
-        <v>168</v>
-      </c>
-      <c r="J75" t="s">
-        <v>13</v>
-      </c>
-      <c r="K75" t="s">
-        <v>12</v>
-      </c>
-      <c r="L75">
-        <v>506001</v>
-      </c>
-    </row>
-    <row r="76" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A76">
-        <v>9542895197</v>
-      </c>
-      <c r="B76" t="s">
-        <v>169</v>
-      </c>
-      <c r="C76">
-        <v>516</v>
-      </c>
-      <c r="D76" t="s">
-        <v>10</v>
-      </c>
-      <c r="G76">
-        <v>2379</v>
-      </c>
-      <c r="H76">
-        <v>46201</v>
-      </c>
-      <c r="I76" t="s">
-        <v>170</v>
-      </c>
-      <c r="J76" t="s">
-        <v>171</v>
-      </c>
-      <c r="K76" t="s">
-        <v>12</v>
-      </c>
-      <c r="L76">
-        <v>502103</v>
-      </c>
-    </row>
-    <row r="77" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A77">
-        <v>7893800980</v>
-      </c>
-      <c r="B77" t="s">
-        <v>172</v>
-      </c>
-      <c r="C77">
-        <v>520</v>
-      </c>
-      <c r="D77" t="s">
-        <v>10</v>
-      </c>
-      <c r="G77">
-        <v>2380</v>
-      </c>
-      <c r="H77">
-        <v>46201</v>
-      </c>
-      <c r="I77" t="s">
-        <v>173</v>
-      </c>
-      <c r="J77" t="s">
-        <v>11</v>
-      </c>
-      <c r="K77" t="s">
-        <v>12</v>
-      </c>
-      <c r="L77">
-        <v>506002</v>
-      </c>
-    </row>
-    <row r="78" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A78">
-        <v>9849212083</v>
-      </c>
-      <c r="B78" t="s">
-        <v>174</v>
-      </c>
-      <c r="C78">
-        <v>3201</v>
-      </c>
-      <c r="D78" t="s">
-        <v>10</v>
-      </c>
-      <c r="G78">
-        <v>2388</v>
-      </c>
-      <c r="H78">
-        <v>46202</v>
-      </c>
-      <c r="I78" t="s">
-        <v>175</v>
-      </c>
-      <c r="J78" t="s">
-        <v>13</v>
-      </c>
-      <c r="K78" t="s">
-        <v>12</v>
-      </c>
-      <c r="L78">
-        <v>506001</v>
-      </c>
-    </row>
-    <row r="79" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A79">
-        <v>8500288366</v>
-      </c>
-      <c r="B79" t="s">
-        <v>176</v>
-      </c>
-      <c r="C79">
-        <v>516</v>
-      </c>
-      <c r="D79" t="s">
-        <v>10</v>
-      </c>
-      <c r="G79">
-        <v>2389</v>
-      </c>
-      <c r="H79">
-        <v>46202</v>
-      </c>
-      <c r="I79" t="s">
-        <v>177</v>
-      </c>
-      <c r="J79" t="s">
-        <v>13</v>
-      </c>
-      <c r="K79" t="s">
-        <v>12</v>
-      </c>
-      <c r="L79">
-        <v>506001</v>
-      </c>
-    </row>
-    <row r="80" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A80">
-        <v>8500288366</v>
-      </c>
-      <c r="B80" t="s">
-        <v>178</v>
-      </c>
-      <c r="C80">
-        <v>1116</v>
-      </c>
-      <c r="D80" t="s">
-        <v>10</v>
-      </c>
-      <c r="G80">
-        <v>2387</v>
-      </c>
-      <c r="H80">
-        <v>46202</v>
-      </c>
-      <c r="I80" t="s">
-        <v>179</v>
-      </c>
-      <c r="J80" t="s">
-        <v>13</v>
-      </c>
-      <c r="K80" t="s">
-        <v>12</v>
-      </c>
-      <c r="L80">
-        <v>506001</v>
-      </c>
-    </row>
-    <row r="81" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A81">
-        <v>9032375368</v>
-      </c>
-      <c r="B81" t="s">
-        <v>180</v>
-      </c>
-      <c r="C81">
-        <v>516</v>
-      </c>
-      <c r="D81" t="s">
-        <v>10</v>
-      </c>
-      <c r="G81">
-        <v>2386</v>
-      </c>
-      <c r="H81">
-        <v>46202</v>
-      </c>
-      <c r="I81" t="s">
-        <v>181</v>
-      </c>
-      <c r="J81" t="s">
-        <v>11</v>
-      </c>
-      <c r="K81" t="s">
-        <v>12</v>
-      </c>
-      <c r="L81">
-        <v>506003</v>
-      </c>
-    </row>
-    <row r="82" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A82">
-        <v>9908900558</v>
-      </c>
-      <c r="B82" t="s">
-        <v>21</v>
-      </c>
-      <c r="C82">
-        <v>51000</v>
-      </c>
-      <c r="D82" t="s">
-        <v>10</v>
-      </c>
-      <c r="G82">
-        <v>2385</v>
-      </c>
-      <c r="H82">
-        <v>46202</v>
-      </c>
-      <c r="I82" t="s">
-        <v>22</v>
-      </c>
-      <c r="J82" t="s">
-        <v>13</v>
-      </c>
-      <c r="K82" t="s">
-        <v>12</v>
-      </c>
-      <c r="L82">
-        <v>506001</v>
-      </c>
-    </row>
-    <row r="83" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A83">
-        <v>9866568921</v>
-      </c>
-      <c r="B83" t="s">
-        <v>182</v>
-      </c>
-      <c r="C83">
-        <v>501</v>
-      </c>
-      <c r="D83" t="s">
-        <v>10</v>
-      </c>
-      <c r="G83">
-        <v>2392</v>
-      </c>
-      <c r="H83">
-        <v>46202</v>
-      </c>
-      <c r="I83" t="s">
-        <v>183</v>
-      </c>
-      <c r="J83" t="s">
-        <v>11</v>
-      </c>
-      <c r="K83" t="s">
-        <v>12</v>
-      </c>
-      <c r="L83">
-        <v>506002</v>
-      </c>
-    </row>
-    <row r="84" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A84">
-        <v>9652525448</v>
-      </c>
-      <c r="B84" t="s">
-        <v>184</v>
-      </c>
-      <c r="C84">
-        <v>516</v>
-      </c>
-      <c r="D84" t="s">
-        <v>10</v>
-      </c>
-      <c r="G84">
-        <v>2393</v>
-      </c>
-      <c r="H84">
-        <v>46203</v>
-      </c>
-      <c r="I84" t="s">
-        <v>185</v>
-      </c>
-      <c r="J84" t="s">
-        <v>13</v>
-      </c>
-      <c r="K84" t="s">
-        <v>12</v>
-      </c>
-      <c r="L84">
         <v>506001</v>
       </c>
     </row>

</xml_diff>